<commit_message>
Adapeker: kontrolör düzeltmeleri (kolon/perde çakışmaları, 2 SASKİ ağı, ayak kesişmeleri)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RwXcqZmf9VPBpDgb8LPkn3
</commit_message>
<xml_diff>
--- a/proje/adapeker/ADAPEKER_ISI_KAYBI_YERDEN_ISITMA_HESABI.xlsx
+++ b/proje/adapeker/ADAPEKER_ISI_KAYBI_YERDEN_ISITMA_HESABI.xlsx
@@ -22428,7 +22428,7 @@
         <v/>
       </c>
       <c r="I7" s="504" t="n">
-        <v>104.4</v>
+        <v>103.24</v>
       </c>
       <c r="J7" s="504" t="n">
         <v>2</v>
@@ -22478,7 +22478,7 @@
         <v/>
       </c>
       <c r="I8" s="504" t="n">
-        <v>142.75</v>
+        <v>142.47</v>
       </c>
       <c r="J8" s="504" t="n">
         <v>2</v>
@@ -22578,7 +22578,7 @@
         <v/>
       </c>
       <c r="I10" s="504" t="n">
-        <v>22.17</v>
+        <v>21.53</v>
       </c>
       <c r="J10" s="504" t="n">
         <v>1</v>
@@ -22628,7 +22628,7 @@
         <v/>
       </c>
       <c r="I11" s="504" t="n">
-        <v>26.68</v>
+        <v>26.04</v>
       </c>
       <c r="J11" s="504" t="n">
         <v>1</v>
@@ -22778,7 +22778,7 @@
         <v/>
       </c>
       <c r="I14" s="504" t="n">
-        <v>104.4</v>
+        <v>103.24</v>
       </c>
       <c r="J14" s="504" t="n">
         <v>2</v>
@@ -22828,7 +22828,7 @@
         <v/>
       </c>
       <c r="I15" s="504" t="n">
-        <v>142.75</v>
+        <v>142.47</v>
       </c>
       <c r="J15" s="504" t="n">
         <v>2</v>
@@ -22928,7 +22928,7 @@
         <v/>
       </c>
       <c r="I17" s="504" t="n">
-        <v>22.17</v>
+        <v>21.53</v>
       </c>
       <c r="J17" s="504" t="n">
         <v>1</v>
@@ -22978,7 +22978,7 @@
         <v/>
       </c>
       <c r="I18" s="504" t="n">
-        <v>26.68</v>
+        <v>26.04</v>
       </c>
       <c r="J18" s="504" t="n">
         <v>1</v>
@@ -23128,7 +23128,7 @@
         <v/>
       </c>
       <c r="I21" s="504" t="n">
-        <v>104.4</v>
+        <v>103.24</v>
       </c>
       <c r="J21" s="504" t="n">
         <v>2</v>
@@ -23178,7 +23178,7 @@
         <v/>
       </c>
       <c r="I22" s="504" t="n">
-        <v>142.75</v>
+        <v>142.47</v>
       </c>
       <c r="J22" s="504" t="n">
         <v>2</v>
@@ -23278,7 +23278,7 @@
         <v/>
       </c>
       <c r="I24" s="504" t="n">
-        <v>22.17</v>
+        <v>21.53</v>
       </c>
       <c r="J24" s="504" t="n">
         <v>1</v>
@@ -23328,7 +23328,7 @@
         <v/>
       </c>
       <c r="I25" s="504" t="n">
-        <v>26.68</v>
+        <v>26.04</v>
       </c>
       <c r="J25" s="504" t="n">
         <v>1</v>
@@ -23478,7 +23478,7 @@
         <v/>
       </c>
       <c r="I28" s="504" t="n">
-        <v>104.4</v>
+        <v>103.24</v>
       </c>
       <c r="J28" s="504" t="n">
         <v>2</v>
@@ -23528,7 +23528,7 @@
         <v/>
       </c>
       <c r="I29" s="504" t="n">
-        <v>142.75</v>
+        <v>142.47</v>
       </c>
       <c r="J29" s="504" t="n">
         <v>2</v>
@@ -23628,7 +23628,7 @@
         <v/>
       </c>
       <c r="I31" s="504" t="n">
-        <v>22.17</v>
+        <v>21.53</v>
       </c>
       <c r="J31" s="504" t="n">
         <v>1</v>
@@ -23678,7 +23678,7 @@
         <v/>
       </c>
       <c r="I32" s="504" t="n">
-        <v>26.68</v>
+        <v>26.04</v>
       </c>
       <c r="J32" s="504" t="n">
         <v>1</v>
@@ -23828,7 +23828,7 @@
         <v/>
       </c>
       <c r="I35" s="504" t="n">
-        <v>104.4</v>
+        <v>103.24</v>
       </c>
       <c r="J35" s="504" t="n">
         <v>2</v>
@@ -23878,7 +23878,7 @@
         <v/>
       </c>
       <c r="I36" s="504" t="n">
-        <v>142.75</v>
+        <v>142.47</v>
       </c>
       <c r="J36" s="504" t="n">
         <v>2</v>
@@ -23978,7 +23978,7 @@
         <v/>
       </c>
       <c r="I38" s="504" t="n">
-        <v>22.17</v>
+        <v>21.53</v>
       </c>
       <c r="J38" s="504" t="n">
         <v>1</v>
@@ -24028,7 +24028,7 @@
         <v/>
       </c>
       <c r="I39" s="504" t="n">
-        <v>26.68</v>
+        <v>26.04</v>
       </c>
       <c r="J39" s="504" t="n">
         <v>1</v>
@@ -24178,7 +24178,7 @@
         <v/>
       </c>
       <c r="I42" s="504" t="n">
-        <v>104.4</v>
+        <v>103.24</v>
       </c>
       <c r="J42" s="504" t="n">
         <v>2</v>
@@ -24228,7 +24228,7 @@
         <v/>
       </c>
       <c r="I43" s="504" t="n">
-        <v>142.75</v>
+        <v>142.47</v>
       </c>
       <c r="J43" s="504" t="n">
         <v>2</v>
@@ -24328,7 +24328,7 @@
         <v/>
       </c>
       <c r="I45" s="504" t="n">
-        <v>22.17</v>
+        <v>21.53</v>
       </c>
       <c r="J45" s="504" t="n">
         <v>1</v>
@@ -24378,7 +24378,7 @@
         <v/>
       </c>
       <c r="I46" s="504" t="n">
-        <v>26.68</v>
+        <v>26.04</v>
       </c>
       <c r="J46" s="504" t="n">
         <v>1</v>
@@ -24582,16 +24582,16 @@
         <v>3</v>
       </c>
       <c r="F6" s="504" t="n">
-        <v>50.04</v>
+        <v>55.13</v>
       </c>
       <c r="G6" s="504" t="n">
         <v>15</v>
       </c>
       <c r="H6" s="504" t="n">
-        <v>1751.5</v>
+        <v>1929.7</v>
       </c>
       <c r="I6" s="504" t="n">
-        <v>249.6</v>
+        <v>278.1</v>
       </c>
     </row>
     <row r="7">
@@ -24619,16 +24619,16 @@
         <v>4</v>
       </c>
       <c r="F7" s="504" t="n">
-        <v>54.35</v>
+        <v>48.1</v>
       </c>
       <c r="G7" s="504" t="n">
         <v>15</v>
       </c>
       <c r="H7" s="504" t="n">
-        <v>1902.4</v>
+        <v>1683.6</v>
       </c>
       <c r="I7" s="504" t="n">
-        <v>271.1</v>
+        <v>242.6</v>
       </c>
     </row>
     <row r="8">
@@ -24656,16 +24656,16 @@
         <v>5</v>
       </c>
       <c r="F8" s="504" t="n">
-        <v>69.67</v>
+        <v>73.59</v>
       </c>
       <c r="G8" s="504" t="n">
         <v>15</v>
       </c>
       <c r="H8" s="504" t="n">
-        <v>2438.3</v>
+        <v>2575.6</v>
       </c>
       <c r="I8" s="504" t="n">
-        <v>507.6</v>
+        <v>537.2</v>
       </c>
     </row>
     <row r="9">
@@ -24693,16 +24693,16 @@
         <v>6</v>
       </c>
       <c r="F9" s="504" t="n">
-        <v>73.08</v>
+        <v>68.89</v>
       </c>
       <c r="G9" s="504" t="n">
         <v>15</v>
       </c>
       <c r="H9" s="504" t="n">
-        <v>2557.8</v>
+        <v>2411</v>
       </c>
       <c r="I9" s="504" t="n">
-        <v>532.4</v>
+        <v>502.8</v>
       </c>
     </row>
     <row r="10">
@@ -24767,13 +24767,13 @@
         <v>8</v>
       </c>
       <c r="F11" s="504" t="n">
-        <v>22.17</v>
+        <v>21.53</v>
       </c>
       <c r="G11" s="504" t="n">
         <v>15</v>
       </c>
       <c r="H11" s="504" t="n">
-        <v>776</v>
+        <v>753.6</v>
       </c>
       <c r="I11" s="504" t="n">
         <v>193.6</v>
@@ -24804,13 +24804,13 @@
         <v>9</v>
       </c>
       <c r="F12" s="504" t="n">
-        <v>26.68</v>
+        <v>26.04</v>
       </c>
       <c r="G12" s="504" t="n">
         <v>15</v>
       </c>
       <c r="H12" s="504" t="n">
-        <v>933.7</v>
+        <v>911.3</v>
       </c>
       <c r="I12" s="504" t="n">
         <v>60</v>
@@ -24915,16 +24915,16 @@
         <v>12</v>
       </c>
       <c r="F15" s="504" t="n">
-        <v>50.04</v>
+        <v>55.13</v>
       </c>
       <c r="G15" s="504" t="n">
         <v>15</v>
       </c>
       <c r="H15" s="504" t="n">
-        <v>1751.5</v>
+        <v>1929.7</v>
       </c>
       <c r="I15" s="504" t="n">
-        <v>249.6</v>
+        <v>278.1</v>
       </c>
     </row>
     <row r="16">
@@ -24952,16 +24952,16 @@
         <v>13</v>
       </c>
       <c r="F16" s="504" t="n">
-        <v>54.35</v>
+        <v>48.1</v>
       </c>
       <c r="G16" s="504" t="n">
         <v>15</v>
       </c>
       <c r="H16" s="504" t="n">
-        <v>1902.4</v>
+        <v>1683.6</v>
       </c>
       <c r="I16" s="504" t="n">
-        <v>271.1</v>
+        <v>242.6</v>
       </c>
     </row>
     <row r="17">
@@ -24989,16 +24989,16 @@
         <v>14</v>
       </c>
       <c r="F17" s="504" t="n">
-        <v>69.67</v>
+        <v>73.59</v>
       </c>
       <c r="G17" s="504" t="n">
         <v>15</v>
       </c>
       <c r="H17" s="504" t="n">
-        <v>2438.3</v>
+        <v>2575.6</v>
       </c>
       <c r="I17" s="504" t="n">
-        <v>507.6</v>
+        <v>537.2</v>
       </c>
     </row>
     <row r="18">
@@ -25026,16 +25026,16 @@
         <v>15</v>
       </c>
       <c r="F18" s="504" t="n">
-        <v>73.08</v>
+        <v>68.89</v>
       </c>
       <c r="G18" s="504" t="n">
         <v>15</v>
       </c>
       <c r="H18" s="504" t="n">
-        <v>2557.8</v>
+        <v>2411</v>
       </c>
       <c r="I18" s="504" t="n">
-        <v>532.4</v>
+        <v>502.8</v>
       </c>
     </row>
     <row r="19">
@@ -25100,13 +25100,13 @@
         <v>17</v>
       </c>
       <c r="F20" s="504" t="n">
-        <v>22.17</v>
+        <v>21.53</v>
       </c>
       <c r="G20" s="504" t="n">
         <v>15</v>
       </c>
       <c r="H20" s="504" t="n">
-        <v>776</v>
+        <v>753.6</v>
       </c>
       <c r="I20" s="504" t="n">
         <v>193.6</v>
@@ -25137,13 +25137,13 @@
         <v>18</v>
       </c>
       <c r="F21" s="504" t="n">
-        <v>26.68</v>
+        <v>26.04</v>
       </c>
       <c r="G21" s="504" t="n">
         <v>15</v>
       </c>
       <c r="H21" s="504" t="n">
-        <v>933.7</v>
+        <v>911.3</v>
       </c>
       <c r="I21" s="504" t="n">
         <v>60</v>
@@ -25248,16 +25248,16 @@
         <v>21</v>
       </c>
       <c r="F24" s="504" t="n">
-        <v>50.04</v>
+        <v>55.13</v>
       </c>
       <c r="G24" s="504" t="n">
         <v>15</v>
       </c>
       <c r="H24" s="504" t="n">
-        <v>1751.5</v>
+        <v>1929.7</v>
       </c>
       <c r="I24" s="504" t="n">
-        <v>222.2</v>
+        <v>247.6</v>
       </c>
     </row>
     <row r="25">
@@ -25285,16 +25285,16 @@
         <v>22</v>
       </c>
       <c r="F25" s="504" t="n">
-        <v>54.35</v>
+        <v>48.1</v>
       </c>
       <c r="G25" s="504" t="n">
         <v>15</v>
       </c>
       <c r="H25" s="504" t="n">
-        <v>1902.4</v>
+        <v>1683.6</v>
       </c>
       <c r="I25" s="504" t="n">
-        <v>241.3</v>
+        <v>216</v>
       </c>
     </row>
     <row r="26">
@@ -25322,16 +25322,16 @@
         <v>23</v>
       </c>
       <c r="F26" s="504" t="n">
-        <v>69.67</v>
+        <v>73.59</v>
       </c>
       <c r="G26" s="504" t="n">
         <v>15</v>
       </c>
       <c r="H26" s="504" t="n">
-        <v>2438.3</v>
+        <v>2575.6</v>
       </c>
       <c r="I26" s="504" t="n">
-        <v>458.2</v>
+        <v>485</v>
       </c>
     </row>
     <row r="27">
@@ -25359,16 +25359,16 @@
         <v>24</v>
       </c>
       <c r="F27" s="504" t="n">
-        <v>73.08</v>
+        <v>68.89</v>
       </c>
       <c r="G27" s="504" t="n">
         <v>15</v>
       </c>
       <c r="H27" s="504" t="n">
-        <v>2557.8</v>
+        <v>2411</v>
       </c>
       <c r="I27" s="504" t="n">
-        <v>480.7</v>
+        <v>454</v>
       </c>
     </row>
     <row r="28">
@@ -25433,13 +25433,13 @@
         <v>26</v>
       </c>
       <c r="F29" s="504" t="n">
-        <v>22.17</v>
+        <v>21.53</v>
       </c>
       <c r="G29" s="504" t="n">
         <v>15</v>
       </c>
       <c r="H29" s="504" t="n">
-        <v>776</v>
+        <v>753.6</v>
       </c>
       <c r="I29" s="504" t="n">
         <v>170.1</v>
@@ -25470,13 +25470,13 @@
         <v>27</v>
       </c>
       <c r="F30" s="504" t="n">
-        <v>26.68</v>
+        <v>26.04</v>
       </c>
       <c r="G30" s="504" t="n">
         <v>15</v>
       </c>
       <c r="H30" s="504" t="n">
-        <v>933.7</v>
+        <v>911.3</v>
       </c>
       <c r="I30" s="504" t="n">
         <v>46</v>
@@ -25581,16 +25581,16 @@
         <v>30</v>
       </c>
       <c r="F33" s="504" t="n">
-        <v>50.04</v>
+        <v>55.13</v>
       </c>
       <c r="G33" s="504" t="n">
         <v>15</v>
       </c>
       <c r="H33" s="504" t="n">
-        <v>1751.5</v>
+        <v>1929.7</v>
       </c>
       <c r="I33" s="504" t="n">
-        <v>222.2</v>
+        <v>247.6</v>
       </c>
     </row>
     <row r="34">
@@ -25618,16 +25618,16 @@
         <v>31</v>
       </c>
       <c r="F34" s="504" t="n">
-        <v>54.35</v>
+        <v>48.1</v>
       </c>
       <c r="G34" s="504" t="n">
         <v>15</v>
       </c>
       <c r="H34" s="504" t="n">
-        <v>1902.4</v>
+        <v>1683.6</v>
       </c>
       <c r="I34" s="504" t="n">
-        <v>241.3</v>
+        <v>216</v>
       </c>
     </row>
     <row r="35">
@@ -25655,16 +25655,16 @@
         <v>32</v>
       </c>
       <c r="F35" s="504" t="n">
-        <v>69.67</v>
+        <v>73.59</v>
       </c>
       <c r="G35" s="504" t="n">
         <v>15</v>
       </c>
       <c r="H35" s="504" t="n">
-        <v>2438.3</v>
+        <v>2575.6</v>
       </c>
       <c r="I35" s="504" t="n">
-        <v>458.2</v>
+        <v>485</v>
       </c>
     </row>
     <row r="36">
@@ -25692,16 +25692,16 @@
         <v>33</v>
       </c>
       <c r="F36" s="504" t="n">
-        <v>73.08</v>
+        <v>68.89</v>
       </c>
       <c r="G36" s="504" t="n">
         <v>15</v>
       </c>
       <c r="H36" s="504" t="n">
-        <v>2557.8</v>
+        <v>2411</v>
       </c>
       <c r="I36" s="504" t="n">
-        <v>480.7</v>
+        <v>454</v>
       </c>
     </row>
     <row r="37">
@@ -25766,13 +25766,13 @@
         <v>35</v>
       </c>
       <c r="F38" s="504" t="n">
-        <v>22.17</v>
+        <v>21.53</v>
       </c>
       <c r="G38" s="504" t="n">
         <v>15</v>
       </c>
       <c r="H38" s="504" t="n">
-        <v>776</v>
+        <v>753.6</v>
       </c>
       <c r="I38" s="504" t="n">
         <v>170.1</v>
@@ -25803,13 +25803,13 @@
         <v>36</v>
       </c>
       <c r="F39" s="504" t="n">
-        <v>26.68</v>
+        <v>26.04</v>
       </c>
       <c r="G39" s="504" t="n">
         <v>15</v>
       </c>
       <c r="H39" s="504" t="n">
-        <v>933.7</v>
+        <v>911.3</v>
       </c>
       <c r="I39" s="504" t="n">
         <v>46</v>
@@ -25914,16 +25914,16 @@
         <v>39</v>
       </c>
       <c r="F42" s="504" t="n">
-        <v>50.04</v>
+        <v>55.13</v>
       </c>
       <c r="G42" s="504" t="n">
         <v>15</v>
       </c>
       <c r="H42" s="504" t="n">
-        <v>1751.5</v>
+        <v>1929.7</v>
       </c>
       <c r="I42" s="504" t="n">
-        <v>260.8</v>
+        <v>290.5</v>
       </c>
     </row>
     <row r="43">
@@ -25951,16 +25951,16 @@
         <v>40</v>
       </c>
       <c r="F43" s="504" t="n">
-        <v>54.35</v>
+        <v>48.1</v>
       </c>
       <c r="G43" s="504" t="n">
         <v>15</v>
       </c>
       <c r="H43" s="504" t="n">
-        <v>1902.4</v>
+        <v>1683.6</v>
       </c>
       <c r="I43" s="504" t="n">
-        <v>283.2</v>
+        <v>253.5</v>
       </c>
     </row>
     <row r="44">
@@ -25988,16 +25988,16 @@
         <v>41</v>
       </c>
       <c r="F44" s="504" t="n">
-        <v>69.67</v>
+        <v>73.59</v>
       </c>
       <c r="G44" s="504" t="n">
         <v>15</v>
       </c>
       <c r="H44" s="504" t="n">
-        <v>2438.3</v>
+        <v>2575.6</v>
       </c>
       <c r="I44" s="504" t="n">
-        <v>527.7</v>
+        <v>558.5</v>
       </c>
     </row>
     <row r="45">
@@ -26025,16 +26025,16 @@
         <v>42</v>
       </c>
       <c r="F45" s="504" t="n">
-        <v>73.08</v>
+        <v>68.89</v>
       </c>
       <c r="G45" s="504" t="n">
         <v>15</v>
       </c>
       <c r="H45" s="504" t="n">
-        <v>2557.8</v>
+        <v>2411</v>
       </c>
       <c r="I45" s="504" t="n">
-        <v>553.6</v>
+        <v>522.8</v>
       </c>
     </row>
     <row r="46">
@@ -26099,13 +26099,13 @@
         <v>44</v>
       </c>
       <c r="F47" s="504" t="n">
-        <v>22.17</v>
+        <v>21.53</v>
       </c>
       <c r="G47" s="504" t="n">
         <v>15</v>
       </c>
       <c r="H47" s="504" t="n">
-        <v>776</v>
+        <v>753.6</v>
       </c>
       <c r="I47" s="504" t="n">
         <v>200.3</v>
@@ -26136,13 +26136,13 @@
         <v>45</v>
       </c>
       <c r="F48" s="504" t="n">
-        <v>26.68</v>
+        <v>26.04</v>
       </c>
       <c r="G48" s="504" t="n">
         <v>15</v>
       </c>
       <c r="H48" s="504" t="n">
-        <v>933.7</v>
+        <v>911.3</v>
       </c>
       <c r="I48" s="504" t="n">
         <v>64</v>
@@ -26247,16 +26247,16 @@
         <v>48</v>
       </c>
       <c r="F51" s="504" t="n">
-        <v>50.04</v>
+        <v>55.13</v>
       </c>
       <c r="G51" s="504" t="n">
         <v>15</v>
       </c>
       <c r="H51" s="504" t="n">
-        <v>1751.5</v>
+        <v>1929.7</v>
       </c>
       <c r="I51" s="504" t="n">
-        <v>260.8</v>
+        <v>290.5</v>
       </c>
     </row>
     <row r="52">
@@ -26284,16 +26284,16 @@
         <v>49</v>
       </c>
       <c r="F52" s="504" t="n">
-        <v>54.35</v>
+        <v>48.1</v>
       </c>
       <c r="G52" s="504" t="n">
         <v>15</v>
       </c>
       <c r="H52" s="504" t="n">
-        <v>1902.4</v>
+        <v>1683.6</v>
       </c>
       <c r="I52" s="504" t="n">
-        <v>283.2</v>
+        <v>253.5</v>
       </c>
     </row>
     <row r="53">
@@ -26321,16 +26321,16 @@
         <v>50</v>
       </c>
       <c r="F53" s="504" t="n">
-        <v>69.67</v>
+        <v>73.59</v>
       </c>
       <c r="G53" s="504" t="n">
         <v>15</v>
       </c>
       <c r="H53" s="504" t="n">
-        <v>2438.3</v>
+        <v>2575.6</v>
       </c>
       <c r="I53" s="504" t="n">
-        <v>527.7</v>
+        <v>558.5</v>
       </c>
     </row>
     <row r="54">
@@ -26358,16 +26358,16 @@
         <v>51</v>
       </c>
       <c r="F54" s="504" t="n">
-        <v>73.08</v>
+        <v>68.89</v>
       </c>
       <c r="G54" s="504" t="n">
         <v>15</v>
       </c>
       <c r="H54" s="504" t="n">
-        <v>2557.8</v>
+        <v>2411</v>
       </c>
       <c r="I54" s="504" t="n">
-        <v>553.6</v>
+        <v>522.8</v>
       </c>
     </row>
     <row r="55">
@@ -26432,13 +26432,13 @@
         <v>53</v>
       </c>
       <c r="F56" s="504" t="n">
-        <v>22.17</v>
+        <v>21.53</v>
       </c>
       <c r="G56" s="504" t="n">
         <v>15</v>
       </c>
       <c r="H56" s="504" t="n">
-        <v>776</v>
+        <v>753.6</v>
       </c>
       <c r="I56" s="504" t="n">
         <v>200.3</v>
@@ -26469,13 +26469,13 @@
         <v>54</v>
       </c>
       <c r="F57" s="504" t="n">
-        <v>26.68</v>
+        <v>26.04</v>
       </c>
       <c r="G57" s="504" t="n">
         <v>15</v>
       </c>
       <c r="H57" s="504" t="n">
-        <v>933.7</v>
+        <v>911.3</v>
       </c>
       <c r="I57" s="504" t="n">
         <v>64</v>

</xml_diff>